<commit_message>
Altura por modelo: reconocer talles Short/Long
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DeD19EhRTR4Uun6x1jR1x
</commit_message>
<xml_diff>
--- a/docs/asesor_criterios.xlsx
+++ b/docs/asesor_criterios.xlsx
@@ -23599,12 +23599,20 @@
           <t>Short</t>
         </is>
       </c>
-      <c r="E147" s="9" t="n"/>
-      <c r="F147" s="9" t="n"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" s="9" t="inlineStr">
-        <is>
-          <t>COMPLETAR (no está en la guía)</t>
+      <c r="E147" s="6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F147" s="6" t="n">
+        <v>175</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Guía Marin 2022 (PDF)</t>
+        </is>
+      </c>
+      <c r="H147" s="6" t="inlineStr">
+        <is>
+          <t>Completo</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -23632,12 +23640,20 @@
           <t>Long</t>
         </is>
       </c>
-      <c r="E148" s="9" t="n"/>
-      <c r="F148" s="9" t="n"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" s="9" t="inlineStr">
-        <is>
-          <t>COMPLETAR (no está en la guía)</t>
+      <c r="E148" s="6" t="n">
+        <v>170</v>
+      </c>
+      <c r="F148" s="6" t="n">
+        <v>196</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Guía Marin 2022 (PDF)</t>
+        </is>
+      </c>
+      <c r="H148" s="6" t="inlineStr">
+        <is>
+          <t>Completo</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">

</xml_diff>